<commit_message>
new changes on 12/6/2026
</commit_message>
<xml_diff>
--- a/Testdata/ExcelData.xlsx
+++ b/Testdata/ExcelData.xlsx
@@ -11,13 +11,14 @@
     <sheet sheetId="2" name="MultipleData" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Credentials" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="sheet5" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="govind" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>hello all</t>
   </si>
@@ -95,6 +96,9 @@
   </si>
   <si>
     <t>shoes rack metal</t>
+  </si>
+  <si>
+    <t>shoes</t>
   </si>
 </sst>
 </file>
@@ -617,6 +621,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>